<commit_message>
docs: close VID-03, VID-04 and VID-06 in the backlog
Open count drops to 6 (P1: 1, P2: 4, SEC: 1). VID-06's acceptance criterion is
rewritten to what is actually achievable — audio covering the full video plus a
warning — since no fix can invent 5.2s of narration.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SPRINT_BACKLOG.xlsx
+++ b/SPRINT_BACKLOG.xlsx
@@ -635,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E22"/>
+  <dimension ref="B2:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -761,10 +761,10 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="9" t="n">
         <v>4</v>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>1</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>VID-03 + VID-04 + VID-06 — cùng một họ 'tiếng và hình lệch độ dài', nên sửa chung một lượt</t>
+          <t>VID-07 — bỏ map audio cứng, B-roll mới vào được bản remix</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>VID-07 — bỏ map audio cứng, B-roll mới vào được bản remix</t>
+          <t>SCR-01 — quyết định gỡ hay thay TikTok bằng YouTube Shorts</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>SCR-01 — quyết định gỡ hay thay TikTok bằng YouTube Shorts</t>
+          <t>SEC-01 — rotate key, độc lập với mọi việc khác</t>
         </is>
       </c>
     </row>
@@ -850,16 +850,6 @@
         <v>4</v>
       </c>
       <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>SEC-01 — rotate key, độc lập với mọi việc khác</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Chạy kiểm thử 4 pipeline nặng AI còn lại (xem sheet Ghi chú)</t>
         </is>
@@ -1131,9 +1121,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>Đang mở</t>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Đã đóng</t>
         </is>
       </c>
       <c r="D5" s="22" t="inlineStr">
@@ -1163,15 +1153,19 @@
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>Đệm im lặng cho audio đủ độ dài video (apad) và bỏ -shortest, hoặc chỉ dùng -shortest khi audio dài hơn hình</t>
+          <t>Thêm mux_audio_to_video() trong ffmpeg_utils: đệm audio bằng apad rồi cắt đúng độ dài video, không bao giờ cắt hình theo tiếng</t>
         </is>
       </c>
       <c r="J5" s="22" t="inlineStr">
         <is>
-          <t>Video ra luôn bằng độ dài nguồn (sai số &lt; 0.1s) với lời đọc dài, ngắn và rất ngắn</t>
-        </is>
-      </c>
-      <c r="K5" s="23" t="inlineStr"/>
+          <t>Video ra luôn bằng độ dài nguồn. ĐO ĐƯỢC: 8.00s hình / 8.00s tiếng (trước là 6.42s)</t>
+        </is>
+      </c>
+      <c r="K5" s="23" t="inlineStr">
+        <is>
+          <t>33ea93d</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="78" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
@@ -1184,9 +1178,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>Đang mở</t>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Đã đóng</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
@@ -1206,25 +1200,29 @@
       </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
-          <t>Bước nối hook với video đã polish không đồng bộ độ dài hai luồng</t>
+          <t>Track im lặng của hook dựng ở 24kHz mono trong khi body 48kHz stereo; concat demuxer KHÔNG resample nên audio body phát ở nửa tốc độ, kéo timeline lên gần gấp đôi</t>
         </is>
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
-          <t>modes/polish/polish_pipeline.py · core/concat_helper.py</t>
+          <t>modes/pro_editor/hook_variant_generator.py :: prepend_hook_to_body</t>
         </is>
       </c>
       <c r="I6" s="19" t="inlineStr">
         <is>
-          <t>Sau khi nối thì cắt hoặc đệm cho hai luồng khớp; thêm bước kiểm tra cuối bằng ffprobe</t>
+          <t>Dựng track im lặng theo đúng sample rate + số kênh của body, ép -ar/-ac ở đầu ra concat, thêm chốt chặn cắt cho khớp nếu vẫn lệch &gt; 0.2s</t>
         </is>
       </c>
       <c r="J6" s="19" t="inlineStr">
         <is>
-          <t>Mọi file xuất ra có |video − audio| &lt; 0.2s</t>
-        </is>
-      </c>
-      <c r="K6" s="20" t="inlineStr"/>
+          <t>Mọi file xuất ra có |hình − tiếng| &lt; 0.2s. ĐO ĐƯỢC: 11.00s hình / 11.02s tiếng cho cả 3 bản</t>
+        </is>
+      </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>33ea93d</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="21" t="inlineStr">
@@ -1237,9 +1235,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>Đang mở</t>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Đã đóng</t>
         </is>
       </c>
       <c r="D7" s="22" t="inlineStr">
@@ -1269,15 +1267,19 @@
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>Dùng chung giải pháp với VID-03 — đệm im lặng tới hết video hoặc để nhạc nền lấp phần trống</t>
+          <t>Dùng chung mux_audio_to_video() với VID-03 nên luồng tiếng phủ hết video; cảnh báo rõ khi khoảng trống &gt; 2s để người dùng viết kịch bản dài hơn hoặc thêm nhạc nền</t>
         </is>
       </c>
       <c r="J7" s="22" t="inlineStr">
         <is>
-          <t>Không có đoạn im lặng &gt; 1s ở cuối khi kịch bản ngắn</t>
-        </is>
-      </c>
-      <c r="K7" s="23" t="inlineStr"/>
+          <t>SỬA TIÊU CHÍ: không thể bịa lời đọc để lấp 5.2s, và kéo giãn tới mức đó thì giọng vỡ. Nay yêu cầu: luồng tiếng phủ hết video (lệch &lt; 0.3s) + có cảnh báo. ĐO ĐƯỢC: 8.00s / 8.00s</t>
+        </is>
+      </c>
+      <c r="K7" s="23" t="inlineStr">
+        <is>
+          <t>33ea93d</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="16" t="inlineStr">

</xml_diff>

<commit_message>
docs: close VID-07, no P0 or P1 issues left open
Records the corrected root cause: the failing map pointed at the segment, not
the B-roll clip, and pinning the B-roll audio surfaced a second layer where
segments carried the TTS file's 24kHz mono into a concat that does not resample.

Open count drops to 5, all P2 or security.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SPRINT_BACKLOG.xlsx
+++ b/SPRINT_BACKLOG.xlsx
@@ -635,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E21"/>
+  <dimension ref="B2:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -761,10 +761,10 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>VID-07 — bỏ map audio cứng, B-roll mới vào được bản remix</t>
+          <t>SCR-01 — quyết định gỡ hay thay TikTok bằng YouTube Shorts</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>SCR-01 — quyết định gỡ hay thay TikTok bằng YouTube Shorts</t>
+          <t>SEC-01 — rotate key, độc lập với mọi việc khác</t>
         </is>
       </c>
     </row>
@@ -840,16 +840,6 @@
         <v>3</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>SEC-01 — rotate key, độc lập với mọi việc khác</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Chạy kiểm thử 4 pipeline nặng AI còn lại (xem sheet Ghi chú)</t>
         </is>
@@ -1292,9 +1282,9 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>Đang mở</t>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Đã đóng</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
@@ -1314,25 +1304,29 @@
       </c>
       <c r="G8" s="19" t="inlineStr">
         <is>
-          <t>Map cứng -map 1:a:0 trong khi clip B-roll tải từ Pexels/Pixabay/YouTube thường không có luồng audio; lỗi bị nuốt rồi lặng lẽ dùng bản gốc</t>
+          <t>SỬA LẠI NGUYÊN NHÂN: -map 1:a:0 trỏ vào SEGMENT chứ không phải B-roll. full_remix đã tước audio gốc nên segment có thể không còn luồng tiếng -&gt; ffmpeg thoát, lỗi bị nuốt, mọi segment lặng lẽ quay về bản gốc. Ghim clip B-roll về 48kHz lại làm lộ tầng thứ hai: segment cắt từ video lồng tiếng mang 24kHz mono theo file TTS, concat demuxer không resample nên 12.00s hình chỉ còn 9.02s tiếng</t>
         </is>
       </c>
       <c r="H8" s="20" t="inlineStr">
         <is>
-          <t>modes/full_remix/remix_cut_generator.py :: _mux_broll_with_audio</t>
+          <t>modes/full_remix/remix_cut_generator.py :: _mux_broll_with_audio · core/ffmpeg_utils.py :: normalize_segment_cfr</t>
         </is>
       </c>
       <c r="I8" s="19" t="inlineStr">
         <is>
-          <t>Kiểm tra clip có audio bằng ffprobe trước khi map, hoặc dùng -map 1:a:0? để ffmpeg tự bỏ qua</t>
+          <t>Thiếu tiếng thì lấy im lặng làm input 1 để giữ nguyên chỉ số map; và chuẩn hoá tận gốc: normalize_segment_cfr (mọi concat đều đi qua) nay ép audio về 48kHz stereo, tự cấp luồng im lặng cho clip câm</t>
         </is>
       </c>
       <c r="J8" s="19" t="inlineStr">
         <is>
-          <t>Log không còn dòng 'B-roll mux failed' và bản remix thực sự có cảnh B-roll</t>
-        </is>
-      </c>
-      <c r="K8" s="20" t="inlineStr"/>
+          <t>Hết dòng 'B-roll mux failed', bản remix có cảnh B-roll thật. ĐO ĐƯỢC: 2/4 segment được thay, remix 12.03s hình / 12.10s tiếng (trước 12.00 / 9.02)</t>
+        </is>
+      </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>8dbc382</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="78" customHeight="1">
       <c r="A9" s="21" t="inlineStr">

</xml_diff>